<commit_message>
habitas générés ok !
</commit_message>
<xml_diff>
--- a/scripts/pokomons.xlsx
+++ b/scripts/pokomons.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="186">
   <si>
     <t>LVL</t>
   </si>
@@ -121,6 +121,9 @@
     <t>TODO</t>
   </si>
   <si>
+    <t>TODO SPAWN</t>
+  </si>
+  <si>
     <t>EV</t>
   </si>
   <si>
@@ -190,6 +193,9 @@
     <t>cby:forge_side</t>
   </si>
   <si>
+    <t>TODO STRUCTURE ET SPAWN</t>
+  </si>
+  <si>
     <t>STRUCTURE</t>
   </si>
   <si>
@@ -271,7 +277,7 @@
     <t>need silktouch</t>
   </si>
   <si>
-    <t>lapiz_ore</t>
+    <t>lapis_ore</t>
   </si>
   <si>
     <t>redstone_ore</t>
@@ -340,10 +346,10 @@
     <t>wool</t>
   </si>
   <si>
-    <t>pinap_berry_tree</t>
-  </si>
-  <si>
-    <t>weaper_berry_tree</t>
+    <t>cb:pinap_berry</t>
+  </si>
+  <si>
+    <t>cb:wepear_berry</t>
   </si>
   <si>
     <t>miltank</t>
@@ -379,7 +385,7 @@
     <t>cby:tapis_poison</t>
   </si>
   <si>
-    <t>lilypad</t>
+    <t>lily_pad</t>
   </si>
   <si>
     <t>mangrove_roots</t>
@@ -466,13 +472,13 @@
     <t>seeds</t>
   </si>
   <si>
-    <t>cb:oran_berry_tree</t>
-  </si>
-  <si>
-    <t>cb:cherry_berry_tree</t>
-  </si>
-  <si>
-    <t>cb:chesto_berry_tree</t>
+    <t>cb:oran_berry</t>
+  </si>
+  <si>
+    <t>cb:cherry_berry</t>
+  </si>
+  <si>
+    <t>cb:chesto_berry</t>
   </si>
   <si>
     <t>EV16</t>
@@ -1184,20 +1190,14 @@
         <v>34</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="K5" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>34</v>
-      </c>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
       <c r="M5" s="12"/>
       <c r="N5" s="12"/>
       <c r="O5" s="12"/>
@@ -1220,10 +1220,10 @@
         <v>40.0</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
@@ -1231,7 +1231,7 @@
       <c r="H6" s="12"/>
       <c r="I6" s="15"/>
       <c r="J6" s="14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
@@ -1255,10 +1255,10 @@
         <v>40.0</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
@@ -1266,7 +1266,7 @@
       <c r="H7" s="12"/>
       <c r="I7" s="15"/>
       <c r="J7" s="14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
@@ -1290,33 +1290,33 @@
         <v>10.0</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="9"/>
       <c r="J8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
@@ -1337,10 +1337,10 @@
         <v>20.0</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>19</v>
@@ -1349,18 +1349,18 @@
         <v>20</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H9" s="8"/>
       <c r="I9" s="9"/>
       <c r="J9" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="11"/>
@@ -1382,10 +1382,10 @@
         <v>30.0</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>33</v>
@@ -1394,39 +1394,39 @@
         <v>20</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H10" s="8"/>
       <c r="I10" s="9"/>
       <c r="J10" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T10" s="12"/>
       <c r="U10" s="12"/>
@@ -1438,22 +1438,22 @@
         <v/>
       </c>
       <c r="B11" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="15"/>
@@ -1480,27 +1480,27 @@
         <v>20.0</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H12" s="12"/>
+        <v>58</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>59</v>
+      </c>
       <c r="I12" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="J12" s="14" t="s">
-        <v>34</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="J12" s="14"/>
       <c r="K12" s="12"/>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
@@ -1523,10 +1523,10 @@
         <v>20.0</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="12"/>
@@ -1534,19 +1534,19 @@
       <c r="H13" s="12"/>
       <c r="I13" s="15"/>
       <c r="J13" s="17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N13" s="14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
@@ -1563,28 +1563,28 @@
         <v/>
       </c>
       <c r="B14" s="14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="H14" s="12"/>
+        <v>67</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>68</v>
+      </c>
       <c r="I14" s="15"/>
-      <c r="J14" s="14" t="s">
-        <v>66</v>
-      </c>
+      <c r="J14" s="14"/>
       <c r="K14" s="12"/>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
@@ -1607,24 +1607,24 @@
         <v>20.0</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
       <c r="J15" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
@@ -1648,30 +1648,30 @@
         <v>20.0</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H16" s="7"/>
       <c r="I16" s="9"/>
       <c r="J16" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="M16" s="10"/>
       <c r="N16" s="11"/>
@@ -1690,22 +1690,22 @@
         <v/>
       </c>
       <c r="B17" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H17" s="8"/>
       <c r="I17" s="9"/>
@@ -1732,24 +1732,24 @@
         <v>20.0</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="15"/>
       <c r="J18" s="14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
@@ -1773,29 +1773,29 @@
         <v>20.0</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H19" s="12"/>
       <c r="I19" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K19" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L19" s="12"/>
       <c r="M19" s="12"/>
@@ -1818,51 +1818,51 @@
         <v>20.0</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H20" s="12"/>
       <c r="I20" s="15"/>
       <c r="J20" s="14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="O20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R20" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="S20" s="14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="T20" s="12"/>
       <c r="U20" s="12"/>
@@ -1877,24 +1877,24 @@
         <v>30.0</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H21" s="7"/>
       <c r="I21" s="9"/>
       <c r="J21" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K21" s="10"/>
       <c r="L21" s="10"/>
@@ -1918,37 +1918,37 @@
         <v>40.0</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>25</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
       <c r="I22" s="9"/>
       <c r="J22" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N22" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O22" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P22" s="11"/>
       <c r="Q22" s="11"/>
@@ -1967,30 +1967,30 @@
         <v>20.0</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="H23" s="8"/>
+        <v>106</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>59</v>
+      </c>
       <c r="I23" s="20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="K23" s="14" t="s">
-        <v>34</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="K23" s="14"/>
       <c r="L23" s="14"/>
       <c r="M23" s="14"/>
       <c r="N23" s="12"/>
@@ -2012,25 +2012,25 @@
         <v>10.0</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="9"/>
       <c r="J24" s="21" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K24" s="21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L24" s="10"/>
       <c r="M24" s="10"/>
@@ -2053,37 +2053,37 @@
         <v>20.0</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
       <c r="J25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="P25" s="11"/>
       <c r="Q25" s="11"/>
@@ -2102,20 +2102,20 @@
         <v>30.0</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F26" s="19"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="20"/>
       <c r="J26" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
@@ -2139,38 +2139,38 @@
         <v>40.0</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D27" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>114</v>
       </c>
       <c r="F27" s="19"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="20"/>
       <c r="J27" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M27" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="Q27" s="11"/>
       <c r="R27" s="11"/>
@@ -2188,10 +2188,10 @@
         <v>10.0</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>19</v>
@@ -2200,15 +2200,15 @@
         <v>23</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H28" s="12"/>
       <c r="I28" s="15"/>
       <c r="J28" s="17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L28" s="12"/>
       <c r="M28" s="12"/>
@@ -2231,10 +2231,10 @@
         <v>20.0</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E29" s="14" t="s">
         <v>19</v>
@@ -2243,24 +2243,24 @@
         <v>20</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H29" s="12"/>
       <c r="I29" s="15"/>
       <c r="J29" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K29" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="O29" s="12"/>
       <c r="P29" s="12"/>
@@ -2277,13 +2277,13 @@
         <v/>
       </c>
       <c r="B30" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E30" s="12"/>
       <c r="F30" s="12"/>
@@ -2291,16 +2291,16 @@
       <c r="H30" s="12"/>
       <c r="I30" s="15"/>
       <c r="J30" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K30" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N30" s="12"/>
       <c r="O30" s="12"/>
@@ -2318,13 +2318,13 @@
         <v/>
       </c>
       <c r="B31" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E31" s="12"/>
       <c r="F31" s="12"/>
@@ -2351,22 +2351,22 @@
         <v/>
       </c>
       <c r="B32" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E32" s="14" t="s">
         <v>19</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="15"/>
@@ -2393,10 +2393,10 @@
         <v>20.0</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
@@ -2426,10 +2426,10 @@
         <v>30.0</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>34</v>
@@ -2467,50 +2467,50 @@
         <v>10.0</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I35" s="9"/>
       <c r="J35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="M35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="R35" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="S35" s="11"/>
       <c r="T35" s="12"/>
@@ -2526,27 +2526,27 @@
         <v>20.0</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
       <c r="J36" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L36" s="10"/>
       <c r="M36" s="10"/>
@@ -2569,30 +2569,30 @@
         <v>10.0</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="9"/>
-      <c r="J37" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="K37" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="L37" s="10" t="s">
+      <c r="J37" s="21" t="s">
         <v>152</v>
+      </c>
+      <c r="K37" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="L37" s="21" t="s">
+        <v>154</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="11"/>
@@ -2611,22 +2611,22 @@
         <v/>
       </c>
       <c r="B38" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
@@ -2652,7 +2652,7 @@
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E39" s="7"/>
       <c r="F39" s="19"/>
@@ -2684,10 +2684,10 @@
       <c r="C40" s="18"/>
       <c r="D40" s="13"/>
       <c r="E40" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
@@ -2717,10 +2717,10 @@
       <c r="C41" s="18"/>
       <c r="D41" s="13"/>
       <c r="E41" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
@@ -2750,10 +2750,10 @@
       <c r="C42" s="18"/>
       <c r="D42" s="13"/>
       <c r="E42" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
@@ -2783,16 +2783,16 @@
       <c r="C43" s="18"/>
       <c r="D43" s="13"/>
       <c r="E43" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="K43" s="10"/>
       <c r="L43" s="10"/>
@@ -2815,10 +2815,10 @@
       <c r="C44" s="18"/>
       <c r="D44" s="13"/>
       <c r="E44" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
@@ -2845,10 +2845,10 @@
       <c r="C45" s="18"/>
       <c r="D45" s="13"/>
       <c r="E45" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
@@ -2875,10 +2875,10 @@
       <c r="C46" s="18"/>
       <c r="D46" s="13"/>
       <c r="E46" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
@@ -2905,10 +2905,10 @@
       <c r="C47" s="18"/>
       <c r="D47" s="13"/>
       <c r="E47" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
@@ -2935,10 +2935,10 @@
       <c r="C48" s="18"/>
       <c r="D48" s="13"/>
       <c r="E48" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
@@ -2965,10 +2965,10 @@
       <c r="C49" s="18"/>
       <c r="D49" s="13"/>
       <c r="E49" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
@@ -2995,10 +2995,10 @@
       <c r="C50" s="18"/>
       <c r="D50" s="13"/>
       <c r="E50" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
@@ -3025,10 +3025,10 @@
       <c r="C51" s="18"/>
       <c r="D51" s="13"/>
       <c r="E51" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
@@ -3055,16 +3055,16 @@
       <c r="C52" s="18"/>
       <c r="D52" s="13"/>
       <c r="E52" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="9"/>
       <c r="J52" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="K52" s="10"/>
       <c r="L52" s="10"/>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E53" s="8"/>
       <c r="F53" s="8"/>
@@ -3097,16 +3097,16 @@
       <c r="H53" s="8"/>
       <c r="I53" s="9"/>
       <c r="J53" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L53" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M53" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="N53" s="11"/>
       <c r="O53" s="11"/>
@@ -3128,24 +3128,24 @@
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J54" s="10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="K54" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L54" s="11"/>
       <c r="M54" s="11"/>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="C55" s="24"/>
       <c r="D55" s="14" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E55" s="12"/>
       <c r="F55" s="12"/>
@@ -3199,10 +3199,10 @@
       <c r="C56" s="24"/>
       <c r="D56" s="12"/>
       <c r="E56" s="14" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G56" s="12"/>
       <c r="H56" s="12"/>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="C57" s="14"/>
       <c r="D57" s="14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E57" s="12"/>
       <c r="F57" s="12"/>
@@ -3235,7 +3235,7 @@
       <c r="H57" s="12"/>
       <c r="I57" s="15"/>
       <c r="J57" s="14" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="K57" s="12"/>
       <c r="L57" s="12"/>

</xml_diff>